<commit_message>
docs: finalize analytics deployment and GA4 receipt evidence
</commit_message>
<xml_diff>
--- a/outputs/mission9/02_Tracking_Plan.xlsx
+++ b/outputs/mission9/02_Tracking_Plan.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="이벤트" sheetId="1" r:id="R64273ddcae2d4f31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="속성" sheetId="2" r:id="R811cb94148104ba1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="3" r:id="R69fc47c8cf95449c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UTM" sheetId="4" r:id="R3c405d23685948e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="이벤트" sheetId="1" r:id="R1289e02b4ff34017"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="속성" sheetId="2" r:id="R9281f61ff5ef4e47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="3" r:id="R0863ca5c3b494524"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UTM" sheetId="4" r:id="R9c1466aeab1f4a0a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1354,7 +1354,7 @@
         <x:v>단위 테스트 통과</x:v>
       </x:c>
       <x:c r="F18" s="11" t="str">
-        <x:v>계정 미생성</x:v>
+        <x:v>운영 page_view·CTA 실시간 수신</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="62" customHeight="1">
@@ -1371,10 +1371,10 @@
         <x:v>이벤트·속성·사용자 타임라인 일치</x:v>
       </x:c>
       <x:c r="E19" s="10" t="str">
-        <x:v>계정 미생성</x:v>
+        <x:v>US·키·운영 적용</x:v>
       </x:c>
       <x:c r="F19" s="10" t="str">
-        <x:v>미완료</x:v>
+        <x:v>연결 실패; 수신 미확인</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -1391,10 +1391,10 @@
         <x:v>page_view 중복 없음, 캠페인 구분</x:v>
       </x:c>
       <x:c r="E20" s="11" t="str">
-        <x:v>계정 미생성</x:v>
+        <x:v>태그 게시·향상된 측정 해제</x:v>
       </x:c>
       <x:c r="F20" s="11" t="str">
-        <x:v>미완료</x:v>
+        <x:v>실시간 page_view 2·CTA 1 확인; 속성·유입 보고서 대기</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="62" customHeight="1">

</xml_diff>